<commit_message>
Restrict M&A tab to Strategic M&A / PE Buyout deal types
Remove SageSure continuation vehicle (GP-led secondary, no change of
control) and Carbon Underwriting minority growth investment — neither
fits the two allowed deal types. Relabel remaining 8 rows accordingly;
REPAY carried as PE Buyout with non-binding proposal status leading the
notes. Swap myCIO source link to the myCIO sale release confirming a
purchased practice rather than an advisor lift-out.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lgpb2YfdjKwqx2B7EtNxH5
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-07-03.xlsx
+++ b/Weekly_Fintech_Deals_2026-07-03.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Acquisition (carve-out)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Acquisition (tuck-in)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Team/book acquisition</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE-FINTECH FLAG: RIA team/book lift-out, not technology. Closed 30-Jun-26, announced 1-Jul-26. Terms not disclosed; ~$5.3B total client assets are AUM/AUA flow metrics (context only).</t>
+          <t>BORDERLINE-FINTECH FLAG: purchased RIA practice/book, not technology. myCIO SOLD the nine-person Bracaglia team to Clearstead (closed 30-Jun-26, announced 1-Jul-26); terms not disclosed. ~$2.6B AUM + ~$2.7B AUA are flow metrics (context only). Clearstead is majority-owned by Flexpoint Ford.</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Acquisition (100%)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Acquisition (distressed)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Acquisition (PE exit)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -858,17 +858,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Growth equity investment (minority, undisclosed)</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Carbon Underwriting</t>
+          <t>CAWL</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>FTV Capital</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -895,7 +895,7 @@
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Lloyd's delegated-authority underwriting platform with proprietary Graphene data and analytics technology, growing premium from £150M to £471M between 2023 and 2026</t>
+          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -905,14 +905,14 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE-FINTECH FLAG: MGA/underwriting business with a genuine data-platform angle (Graphene). 'Significant' growth equity investment, terms not disclosed; treated as notable strategic-minority investment. £471M premium is GWP (flow metric, context only).</t>
+          <t>Strategic buyout of JV partner: Crédit Agricole acquires Worldline's stake to own 100% of the 2024-created payments JV; Worldline stays on as technology partner. Terms not disclosed.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -922,34 +922,42 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>GP-led continuation vehicle</t>
+          <t>PE Buyout</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>SageSure</t>
+          <t>Repay Holdings (NASDAQ: RPAY)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Flexpoint Ford CV (led by Lexington Partners; Barings, Round2)</t>
+          <t>Forager Capital Management</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+          <t>~1,000</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>3.2x</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>7.8x</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Tech-enabled property insurance managing general underwriter focused on catastrophe-exposed US markets, serving 970,000+ policyholders across 16 states</t>
+          <t>Vertically integrated payments processor for consumer finance and B2B accounts payable/receivable, recently expanded via its $372M KUBRA acquisition closed 1-Jun-26</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -959,128 +967,12 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE STRUCTURE FLAG: &gt;$460M single-asset continuation fund (REPORTED vehicle size, not EV) — GP-led secondary extending Flexpoint Ford's ownership rather than classic M&amp;A. $3.2B written premium is a flow metric (context only, not revenue); no revenue/EBITDA in public record.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>JV stake buyout (to 100%)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>30-Jun-26</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>CAWL</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Crédit Agricole</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Terms not disclosed. Crédit Agricole buys out Worldline's stake to own 100%; Worldline stays on as technology partner supplying acceptance solutions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Take-private proposal (non-binding)</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>29-Jun-26</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Repay Holdings (NASDAQ: RPAY)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Forager Capital Management</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>~1,000</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>3.2x</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>7.8x</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Vertically integrated payments processor for consumer finance and B2B accounts payable/receivable, recently expanded via its $372M KUBRA acquisition closed 1-Jun-26</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Revised unsolicited NON-BINDING proposal of $5.25/sh cash (raised from $4.80 rejected 4-May-26); equity value ~$490M COMPUTED (~93M sh x $5.25); EV ~$1.0B incl. debt REPORTED (press). FY25 REPORTED: revenue $309.3M, adj. EBITDA $128.6M (42% margin). COMPUTED on ~$1.0B EV: EV/Rev = 1,000/309.3 = 3.2x; EV/adj. EBITDA = 1,000/128.6 = 7.8x. Caveat: FY25 financials pre-date KUBRA; multiples approximate.</t>
+          <t>NON-BINDING revised take-private proposal — no agreement signed: Forager (existing stockholder) offered $5.25/sh cash, raised from $4.80 rejected 4-May-26. Equity value ~$490M COMPUTED (~93M sh x $5.25); EV ~$1.0B incl. debt REPORTED (press). FY25 REPORTED: revenue $309.3M, adj. EBITDA $128.6M (42% margin). COMPUTED on ~$1.0B EV: EV/Rev = 1,000/309.3 = 3.2x; EV/adj. EBITDA = 1,000/128.6 = 7.8x. Caveat: FY25 financials pre-date KUBRA; multiples approximate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1090,8 +982,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Apply curated deal list; move Carbon Underwriting to Growth Capital tab
M&A tab now 4 rows (CAWL, FNZ Switzerland, Wealth8, PayEm) per curation
removing non-fintech targets, proposals and deprioritized markets.
Growth Capital tab now 6 rows: Carbon Underwriting joins as an
undisclosed FTV growth equity round (Apiary Capital exit noted); Addi
removed per curation. Second research pass surfaced no additional
in-window qualifying deals.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lgpb2YfdjKwqx2B7EtNxH5
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-07-03.xlsx
+++ b/Weekly_Fintech_Deals_2026-07-03.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -634,12 +634,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Asset &amp; Wealth Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -649,29 +649,37 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>01-Jul-26</t>
+          <t>02-Jul-26</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>myCIO Wealth Partners (Philadelphia team)</t>
+          <t>PayEm</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Clearstead Advisors</t>
+          <t>Top Group Software (via Top Nippando)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+          <t>~4.0</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>0.6x</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>n.m.</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Nine-person Philadelphia advisory team managing ~$2.6B AUM and advising ~$2.7B of institutional assets, joining Clearstead's ~$68B national RIA platform</t>
+          <t>Corporate spend management and procurement SaaS platform for finance teams, sold in a distressed deal after raising ~$27M of equity from Pitango, NFX and Glilot</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -681,19 +689,19 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE-FINTECH FLAG: purchased RIA practice/book, not technology. myCIO SOLD the nine-person Bracaglia team to Clearstead (closed 30-Jun-26, announced 1-Jul-26); terms not disclosed. ~$2.6B AUM + ~$2.7B AUA are flow metrics (context only). Clearstead is majority-owned by Flexpoint Ford.</t>
+          <t>REPORTED: $0.5M for 100% of shares plus buyer commitment to inject up to $3.5M (largely to reduce liabilities); existing equity/options canceled. FY25 REPORTED (Calcalist): revenue NIS 19.1M (~$6.4M), net loss NIS 17.1M (~$5.7M). COMPUTED: EV/Rev = 4.0/6.4 = 0.6x on total-commitment basis ($0.5M + $3.5M); EV/EBITDA n.m. (loss-making).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -703,17 +711,17 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>03-Jul-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>C2FO India Technologies</t>
+          <t>CAWL</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mynd Fintech (M1xchange)</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -725,7 +733,7 @@
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Early-payment and dynamic-discounting platform serving ~140 Indian enterprise clients (roughly half the Nifty 50) and ~200,000 supplier relationships</t>
+          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -735,253 +743,17 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Terms not disclosed. Combined business expected to process ~Rs 60,000 crore (~$7B at Rs 85.5/USD) in annual transactions — flow metric, context only. Carve-out of C2FO's India operations to M1xchange's supply-chain-finance arm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Corporate Financial Function</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>02-Jul-26</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>PayEm</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Top Group Software (via Top Nippando)</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>~4.0</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>0.6x</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>n.m.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Corporate spend management and procurement SaaS platform for finance teams, sold in a distressed deal after raising ~$27M of equity from Pitango, NFX and Glilot</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>REPORTED: $0.5M for 100% of shares plus buyer commitment to inject up to $3.5M (largely to reduce liabilities); existing equity/options canceled. FY25 REPORTED (Calcalist): revenue NIS 19.1M (~$6.4M), net loss NIS 17.1M (~$5.7M). COMPUTED: EV/Rev = 4.0/6.4 = 0.6x on total-commitment basis ($0.5M + $3.5M); EV/EBITDA n.m. (loss-making).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>InsurTech</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>29-Jun-26</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Assured Underwriting Group</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>ANV Group Holdings</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>London-based specialist MGA (founded 1983) underwriting insurance-backed travel bonds and financial-failure cover for 1,600+ tour operators across 10+ European countries</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>BORDERLINE-FINTECH FLAG: traditional specialist MGA rather than insurance software; included as insurance distribution/underwriting M&amp;A. Sold by UK PE firm Mobeus; close expected Q3-26 subject to FCA approval. Terms not disclosed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>30-Jun-26</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>CAWL</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Crédit Agricole</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
           <t>Strategic buyout of JV partner: Crédit Agricole acquires Worldline's stake to own 100% of the 2024-created payments JV; Worldline stays on as technology partner. Terms not disclosed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>PE Buyout</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>29-Jun-26</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Repay Holdings (NASDAQ: RPAY)</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Forager Capital Management</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>~1,000</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>3.2x</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>7.8x</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Vertically integrated payments processor for consumer finance and B2B accounts payable/receivable, recently expanded via its $372M KUBRA acquisition closed 1-Jun-26</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>NON-BINDING revised take-private proposal — no agreement signed: Forager (existing stockholder) offered $5.25/sh cash, raised from $4.80 rejected 4-May-26. Equity value ~$490M COMPUTED (~93M sh x $5.25); EV ~$1.0B incl. debt REPORTED (press). FY25 REPORTED: revenue $309.3M, adj. EBITDA $128.6M (42% margin). COMPUTED on ~$1.0B EV: EV/Rev = 1,000/309.3 = 3.2x; EV/adj. EBITDA = 1,000/128.6 = 7.8x. Caveat: FY25 financials pre-date KUBRA; multiples approximate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1128,33 +900,35 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>01-Jul-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Addi</t>
+          <t>Jota</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Citius and BTG Pactual (GIC, Quona, Monashees, Union Square Ventures, a16z participating)</t>
+          <t>Haun Ventures (HOF Capital, Alter Global, Greyhound Capital participating)</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>185</v>
+      </c>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>BNPL and consumer credit platform serving ~3M customers and 39,000+ merchants in Colombia, profitable for two years and newly approved as a regulated deposit-taking institution</t>
+          <t>AI-powered digital business account and banking platform for Brazilian entrepreneurs and small businesses</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -1164,19 +938,19 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $85M Series D equity; valuation not disclosed. BTG Pactual's first growth-equity deal outside Brazil. Separate $150M JPMorgan-led warehouse facility (Apr-26) is debt — not blended here. Revenue/ARR not disclosed — multiples blank.</t>
+          <t>REPORTED: $30M Series A at $185M post-money valuation. Announcement date per Dealroom deal log (29-Jun-26); some outlets filed 30-Jun — exact day within window but not pinned to a dated press release. Revenue not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1186,25 +960,23 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Jota</t>
+          <t>Nebex</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Haun Ventures (HOF Capital, Alter Global, Greyhound Capital participating)</t>
+          <t>GV (Eniac, 2048 Ventures, Better Tomorrow Ventures et al. participating)</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>185</v>
-      </c>
+      <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AI-powered digital business account and banking platform for Brazilian entrepreneurs and small businesses</t>
+          <t>Exchange-layer market infrastructure connecting space companies with sovereign buyers and deal capital, founded by former Axiom Space CEO Tejpaul Bhatia, banking with J.P. Morgan</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -1214,14 +986,14 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $30M Series A at $185M post-money valuation. Announcement date per Dealroom deal log (29-Jun-26); some outlets filed 30-Jun — exact day within window but not pinned to a dated press release. Revenue not disclosed — multiples blank.</t>
+          <t>BORDERLINE-FINTECH FLAG: capital-markets infrastructure applied to the space economy — fintech angle is the exchange/market plumbing; the end market is the space industry. $30M seed REPORTED; no valuation or revenue disclosed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1231,28 +1003,28 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Nebex</t>
+          <t>LeapXpert</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>GV (Eniac, 2048 Ventures, Better Tomorrow Ventures et al. participating)</t>
+          <t>Riverwood Capital (Portage Ventures participating)</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Exchange-layer market infrastructure connecting space companies with sovereign buyers and deal capital, founded by former Axiom Space CEO Tejpaul Bhatia, banking with J.P. Morgan</t>
+          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1262,7 +1034,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE-FINTECH FLAG: capital-markets infrastructure applied to the space economy — fintech angle is the exchange/market plumbing; the end market is the space industry. $30M seed REPORTED; no valuation or revenue disclosed.</t>
+          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
         </is>
       </c>
     </row>
@@ -1279,28 +1051,28 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>LeapXpert</t>
+          <t>Quantifind</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Riverwood Capital (Portage Ventures participating)</t>
+          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
+          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -1310,45 +1082,47 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
+          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Quantifind</t>
+          <t>Carbon Underwriting</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>200</v>
+          <t>FTV Capital</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
+          <t>Lloyd's delegated-authority underwriting platform with proprietary Graphene data and analytics technology, growing premium from £150M to £471M between 2023 and 2026</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1358,7 +1132,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
+          <t>REPORTED: 'significant' growth equity investment, terms not disclosed; existing investor Apiary Capital exits as part of the deal. £471M premium is GWP (flow metric, context only); revenue/valuation not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Finova/Cubit Labs mortgage-tech acquisition (2-Jul-26)
Surfaced by bottom-up multi-agent sweep (wires, aggregators, vertical
trade press, non-English press) with adversarial date verification;
only candidate of 2 to survive. M&A tab now 5 rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lgpb2YfdjKwqx2B7EtNxH5
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-07-03.xlsx
+++ b/Weekly_Fintech_Deals_2026-07-03.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -747,13 +747,68 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>02-Jul-26</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Cubit Labs</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Finova</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>UK AI startup automating intermediary workflows for mortgage advisers, including document processing and compliance checks, acquired by cloud lending-software platform Finova</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Terms not disclosed. SCALE FLAG: sub-10-person startup founded late 2025 — effectively an acqui-hire of team plus AI product, but a real software asset bought by a strategic (Finova, cloud mortgage/savings/lending software). First disclosed 02-Jul-26 (Mortgage Solutions, Finextra press release).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Taxwire $25M combined seed+Series A to Growth Capital tab
CFO-stack sales-tax automation platform, disclosed 2-Jul-26; basis flag
notes the amount is cumulative across seed and Series A.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lgpb2YfdjKwqx2B7EtNxH5
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-07-03.xlsx
+++ b/Weekly_Fintech_Deals_2026-07-03.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1048,7 +1048,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1058,28 +1058,28 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>02-Jul-26</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>LeapXpert</t>
+          <t>Taxwire</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Riverwood Capital (Portage Ventures participating)</t>
+          <t>Headline, XYZ, Vinyl, Recall Capital, Nomo Ventures (no single lead disclosed)</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>180</v>
+        <v>25</v>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
+          <t>Fully managed AI sales-tax compliance engine automating product tax coding, rate calculation and filing across 22,000+ US jurisdictions and 100+ countries</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
+          <t>BASIS FLAG: $25M is combined Seed + Series A equity disclosed together (REPORTED) — meets the $25M floor only on a cumulative basis. Hundreds of strategic angels (CFOs, controllers, tax specialists) also participated. Outlets ran 30-Jun-2-Jul; in-window on any reading. Revenue/valuation not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
@@ -1106,28 +1106,28 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Quantifind</t>
+          <t>LeapXpert</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
+          <t>Riverwood Capital (Portage Ventures participating)</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
+          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -1137,62 +1137,110 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
+          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Carbon Underwriting</t>
+          <t>Quantifind</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>FTV Capital</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
+          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>200</v>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
+          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Underwriting</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>FTV Capital</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>Lloyd's delegated-authority underwriting platform with proprietary Graphene data and analytics technology, growing premium from £150M to £471M between 2023 and 2026</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>REPORTED: 'significant' growth equity investment, terms not disclosed; existing investor Apiary Capital exits as part of the deal. £471M premium is GWP (flow metric, context only); revenue/valuation not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:L8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1200,6 +1248,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add six deals per explicit direction: SBI/Bitbank, InSoil, Addi, Straiker, Wise/Expatica
M&A tab (+2): SBI Holdings/Bitbank crypto exchange acquisition (signed
24-25 Jun, flagged as pre-window); Wise/Expatica (flagged as pre-window
per Wise's own 18-Jun release date, and as a non-fintech content-business
target).

Growth Capital tab (+3, reinstating Addi): InSoil EUR120M Pollen Street
facility (flagged as debt, not equity); Addi $85M Series D; Straiker
$64M Series A (flagged as horizontal cybersecurity, not fintech-specific).

Every added row carries an explicit notes flag documenting where it
diverges from the stated screening criteria (date window, debt vs
equity, target type) per instruction to include regardless.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lgpb2YfdjKwqx2B7EtNxH5
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-07-03.xlsx
+++ b/Weekly_Fintech_Deals_2026-07-03.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -634,12 +634,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -649,37 +649,29 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>02-Jul-26</t>
+          <t>25-Jun-26</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>PayEm</t>
+          <t>Bitbank</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Top Group Software (via Top Nippando)</t>
+          <t>SBI Holdings</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>~4.0</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>0.6x</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>n.m.</t>
-        </is>
-      </c>
+          <t>289</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Corporate spend management and procurement SaaS platform for finance teams, sold in a distressed deal after raising ~$27M of equity from Pitango, NFX and Glilot</t>
+          <t>Japanese cryptocurrency exchange to become a wholly owned subsidiary of SBI Group, combining with SBI VC Trade to form Japan's largest regulated crypto exchange operator</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -689,19 +681,19 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $0.5M for 100% of shares plus buyer commitment to inject up to $3.5M (largely to reduce liabilities); existing equity/options canceled. FY25 REPORTED (Calcalist): revenue NIS 19.1M (~$6.4M), net loss NIS 17.1M (~$5.7M). COMPUTED: EV/Rev = 4.0/6.4 = 0.6x on total-commitment basis ($0.5M + $3.5M); EV/EBITDA n.m. (loss-making).</t>
+          <t>REPORTED: JPY 46.7bn (~$288.6M/$289M) for 100% of shares. DATE FLAG: basic agreement and share transfer agreement signed 24-25-Jun-26 (Cryptopolitan, The Block, Bitcoin Magazine) — this is BEFORE the stated Sat 27 Jun window; included per explicit instruction despite the date. Structure: SBI acquires founder/individual shares Aug-26, Bitbank buys out corporate holders MIXI and Ceres by end Oct-26, completing full ownership. Combined entity: ~2.92M crypto accounts, ~JPY1.1tn (~$6.8B) AUC — AUC is a flow metric, context only. No revenue/EBITDA disclosed for Bitbank — multiples blank.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -711,29 +703,37 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>02-Jul-26</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>CAWL</t>
+          <t>PayEm</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Crédit Agricole</t>
+          <t>Top Group Software (via Top Nippando)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Undisclosed</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+          <t>~4.0</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>0.6x</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>n.m.</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
+          <t>Corporate spend management and procurement SaaS platform for finance teams, sold in a distressed deal after raising ~$27M of equity from Pitango, NFX and Glilot</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Strategic buyout of JV partner: Crédit Agricole acquires Worldline's stake to own 100% of the 2024-created payments JV; Worldline stays on as technology partner. Terms not disclosed.</t>
+          <t>REPORTED: $0.5M for 100% of shares plus buyer commitment to inject up to $3.5M (largely to reduce liabilities); existing equity/options canceled. FY25 REPORTED (Calcalist): revenue NIS 19.1M (~$6.4M), net loss NIS 17.1M (~$5.7M). COMPUTED: EV/Rev = 4.0/6.4 = 0.6x on total-commitment basis ($0.5M + $3.5M); EV/EBITDA n.m. (loss-making).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -765,17 +765,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>02-Jul-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Cubit Labs</t>
+          <t>CAWL</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Finova</t>
+          <t>Crédit Agricole</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -787,28 +787,138 @@
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>Payment acceptance and acquiring joint venture created in 2024 by Worldline and Crédit Agricole serving French merchants with an integrated payments portal</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Strategic buyout of JV partner: Crédit Agricole acquires Worldline's stake to own 100% of the 2024-created payments JV; Worldline stays on as technology partner. Terms not disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>18-Jun-26</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Expatica</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>~250</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Online resource providing relocation, housing, healthcare, immigration and finance guidance for people living abroad, reaching more than 7 million visits in 2025</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>DOUBLE FLAG: (1) DATE — Wise's own newsroom release and Finextra dated this announcement 18-Jun-26, before the stated Sat 27 Jun window; the fintech.global link (29-Jun) is a roundup repost, not the original announcement. Included per explicit instruction despite the earlier date. (2) TARGET TYPE — Expatica is an expat CONTENT/MEDIA business (country guides, relocation info), not a financial product; the fintech angle is entirely on the acquirer side (Wise folding guides into its money-transfer app). EV ~$250M REPORTED per deal-tracker Windsor Drake — Wise has not confirmed a figure; no target revenue/EBITDA disclosed — multiples blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>02-Jul-26</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Cubit Labs</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Finova</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>UK AI startup automating intermediary workflows for mortgage advisers, including document processing and compliance checks, acquired by cloud lending-software platform Finova</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Terms not disclosed. SCALE FLAG: sub-10-person startup founded late 2025 — effectively an acqui-hire of team plus AI product, but a real software asset bought by a strategic (Finova, cloud mortgage/savings/lending software). First disclosed 02-Jul-26 (Mortgage Solutions, Finextra press release).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -820,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -955,35 +1065,33 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>01-Jul-26</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Jota</t>
+          <t>Addi</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Haun Ventures (HOF Capital, Alter Global, Greyhound Capital participating)</t>
+          <t>Citius and BTG Pactual (GIC, Quona, Monashees, Union Square Ventures, a16z participating)</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>185</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>AI-powered digital business account and banking platform for Brazilian entrepreneurs and small businesses</t>
+          <t>BNPL and consumer credit platform serving ~3M customers and 39,000+ merchants in Colombia, profitable for two years and newly approved as a regulated deposit-taking institution</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
@@ -993,45 +1101,45 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $30M Series A at $185M post-money valuation. Announcement date per Dealroom deal log (29-Jun-26); some outlets filed 30-Jun — exact day within window but not pinned to a dated press release. Revenue not disclosed — multiples blank.</t>
+          <t>REPORTED: $85M Series D equity; valuation not disclosed. BTG Pactual's first growth-equity deal outside Brazil. Separate $150M JPMorgan-led warehouse facility (Apr-26) is debt — not blended here. Revenue/ARR not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nebex</t>
+          <t>InSoil</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>GV (Eniac, 2048 Ventures, Better Tomorrow Ventures et al. participating)</t>
+          <t>Pollen Street Capital</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30</v>
+        <v>130</v>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Exchange-layer market infrastructure connecting space companies with sovereign buyers and deal capital, founded by former Axiom Space CEO Tejpaul Bhatia, banking with J.P. Morgan</t>
+          <t>European climate-finance lender providing mid-term debt to agricultural SMEs transitioning to regenerative farming practices across Europe</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -1041,45 +1149,47 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE-FINTECH FLAG: capital-markets infrastructure applied to the space economy — fintech angle is the exchange/market plumbing; the end market is the space industry. $30M seed REPORTED; no valuation or revenue disclosed.</t>
+          <t>STRUCTURE FLAG: this is DEBT, not equity — a €120M (~$130M at ~1.08 EUR/USD) senior secured CREDIT FACILITY from Pollen Street Capital (backed by an EIF guarantee under InvestEU), not a growth/venture equity raise. Placed on this tab per explicit instruction; 'Amount' reflects facility size, not primary equity proceeds — do not sum with equity rounds on this tab. Founded 2020; 3,500+ agricultural SMEs financed, 15,000+ soil samples collected (flow/operational metrics, context only). No revenue/EBITDA/valuation disclosed — multiples blank. Some sources list HQ as Estonia, one (ArcticStartup) as Lithuania — Estonia used per EU-Startups/BeBeez majority.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>02-Jul-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Taxwire</t>
+          <t>Jota</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Headline, XYZ, Vinyl, Recall Capital, Nomo Ventures (no single lead disclosed)</t>
+          <t>Haun Ventures (HOF Capital, Alter Global, Greyhound Capital participating)</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>185</v>
+      </c>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Fully managed AI sales-tax compliance engine automating product tax coding, rate calculation and filing across 22,000+ US jurisdictions and 100+ countries</t>
+          <t>AI-powered digital business account and banking platform for Brazilian entrepreneurs and small businesses</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1089,14 +1199,14 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>BASIS FLAG: $25M is combined Seed + Series A equity disclosed together (REPORTED) — meets the $25M floor only on a cumulative basis. Hundreds of strategic angels (CFOs, controllers, tax specialists) also participated. Outlets ran 30-Jun-2-Jul; in-window on any reading. Revenue/valuation not disclosed — multiples blank.</t>
+          <t>REPORTED: $30M Series A at $185M post-money valuation. Announcement date per Dealroom deal log (29-Jun-26); some outlets filed 30-Jun — exact day within window but not pinned to a dated press release. Revenue not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1106,28 +1216,28 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>29-Jun-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>LeapXpert</t>
+          <t>Nebex</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Riverwood Capital (Portage Ventures participating)</t>
+          <t>GV (Eniac, 2048 Ventures, Better Tomorrow Ventures et al. participating)</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
+          <t>Exchange-layer market infrastructure connecting space companies with sovereign buyers and deal capital, founded by former Axiom Space CEO Tejpaul Bhatia, banking with J.P. Morgan</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -1137,14 +1247,14 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
+          <t>BORDERLINE-FINTECH FLAG: capital-markets infrastructure applied to the space economy — fintech angle is the exchange/market plumbing; the end market is the space industry. $30M seed REPORTED; no valuation or revenue disclosed.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1154,28 +1264,28 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>29-Jun-26</t>
+          <t>02-Jul-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Quantifind</t>
+          <t>Taxwire</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
+          <t>Headline, XYZ, Vinyl, Recall Capital, Nomo Ventures (no single lead disclosed)</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
+          <t>Fully managed AI sales-tax compliance engine automating product tax coding, rate calculation and filing across 22,000+ US jurisdictions and 100+ countries</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1185,19 +1295,19 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
+          <t>BASIS FLAG: $25M is combined Seed + Series A equity disclosed together (REPORTED) — meets the $25M floor only on a cumulative basis. Hundreds of strategic angels (CFOs, controllers, tax specialists) also participated. Outlets ran 30-Jun-2-Jul; in-window on any reading. Revenue/valuation not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1207,40 +1317,184 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Carbon Underwriting</t>
+          <t>LeapXpert</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>FTV Capital</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Undisclosed</t>
-        </is>
+          <t>Riverwood Capital (Portage Ventures participating)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>180</v>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
+          <t>Governed-communications platform capturing and supervising WhatsApp, iMessage and WeChat business messaging for banks, financial institutions and government agencies</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>REPORTED: $180M growth round. Valuation and revenue/ARR not disclosed — multiples left blank. FS is core segment; government fastest-growing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>29-Jun-26</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Quantifind</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Summit Partners (Citi Ventures, S&amp;P Global, Deloitte, Stephens Group participating)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>AI-native risk intelligence platform (Graphyte) for financial-crime screening and AML used by six of the world's top-10 Tier-1 banks and government agencies</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>REPORTED: $200M growth investment. Valuation and revenue/ARR not disclosed — multiples left blank. Proceeds fund international expansion and Graphyte Agentic Middleware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>29-Jun-26</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Straiker</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Marathon Management Partners, Citi Ventures, Illuminate Financial, Workday Ventures (Bain Capital Ventures, Lightspeed and others participating)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Agentic security platform protecting AI agents deployed inside enterprise environments, grown run-rate revenue more than 15x in under a year</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>NON-FINTECH FLAG: Straiker is a horizontal AI/agentic CYBERSECURITY company, not a financial-services platform — its product secures AI agents generally, not a fintech-specific use case; the brief's own criteria exclude pure cybersecurity. Included per explicit instruction; sector assigned to Financial Info &amp; Analytics as the closest fit given Citi Ventures/Illuminate Financial (fintech-focused) participation, not because the product is finance-specific. REPORTED: $64M Series A, total funding to $85M. Valuation not disclosed — multiples blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Underwriting</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FTV Capital</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>Lloyd's delegated-authority underwriting platform with proprietary Graphene data and analytics technology, growing premium from £150M to £471M between 2023 and 2026</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>REPORTED: 'significant' growth equity investment, terms not disclosed; existing investor Apiary Capital exits as part of the deal. £471M premium is GWP (flow metric, context only); revenue/valuation not disclosed — multiples blank.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1249,6 +1503,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>